<commit_message>
producao: Barretos 2026 v2 — valores reais da produção
Substitui as diárias de referência do orçamento pelo combinado com cada
pessoa, que era a pendência declarada na v1. Entram Larissa (produção adm)
e Danilo (câmeras broadcast, locação de terceiros), e uma terceira entrada
de extras de cinegrafistas.

Bruto 108.500 · imposto 16% 17.360 · líquida 91.140 · saídas 55.400 ·
lucro 35.740 (32,9%). Alimentação durante o evento e hospedagem seguem em
zero — o lucro é antes das duas.

Conferido linha a linha contra o arquivo preenchido pela produção: os onze
totais do RESUMO batem e 0 células com erro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NubHinCg53tN7sLp5QNqJV
</commit_message>
<xml_diff>
--- a/producao/pressupostos/PRESSUPOSTO_REAL_BARRETOS_2026.xlsx
+++ b/producao/pressupostos/PRESSUPOSTO_REAL_BARRETOS_2026.xlsx
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:F56"/>
+  <dimension ref="B1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -785,7 +785,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D13" s="8" t="n"/>
@@ -881,11 +881,21 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="16" t="n"/>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Entrada Extras Cinegrafistas</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="n">
+        <v>27500</v>
+      </c>
       <c r="D19" s="14" t="n"/>
-      <c r="E19" s="15" t="n"/>
-      <c r="F19" s="12" t="n"/>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>A RECEBER</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="B20" s="12" t="n"/>
@@ -902,107 +912,92 @@
       <c r="F21" s="12" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B22" s="12" t="n"/>
+      <c r="C22" s="16" t="n"/>
+      <c r="D22" s="14" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="12" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>TOTAL ENTRADAS (BRUTO)</t>
         </is>
       </c>
-      <c r="C22" s="13">
-        <f>SUM(C17:C21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>IMPOSTO (%)  ← edite aqui se mudar</t>
-        </is>
-      </c>
-      <c r="C23" s="18" t="n">
-        <v>0.16</v>
+      <c r="C23" s="13">
+        <f>SUM(C17:C22)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="12" t="inlineStr">
         <is>
+          <t>IMPOSTO (%)  ← edite aqui se mudar</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="12" t="inlineStr">
+        <is>
           <t>(−) IMPOSTO</t>
         </is>
       </c>
-      <c r="C24" s="13">
-        <f>ROUND(C22*C23,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="19" t="inlineStr">
+      <c r="C25" s="13">
+        <f>ROUND(C23*C24,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="19" t="inlineStr">
         <is>
           <t>(=) ENTRADA LÍQUIDA — é com isso que se paga tudo</t>
         </is>
       </c>
-      <c r="C25" s="20">
-        <f>C22-C24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="10" t="inlineStr">
+      <c r="C26" s="20">
+        <f>C23-C25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>2.  SAÍDAS POR ÁREA — vem sozinho da aba SAÍDAS</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1">
-      <c r="B28" s="11" t="inlineStr">
+    <row r="29" ht="28" customHeight="1">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>ÁREA</t>
         </is>
       </c>
-      <c r="C28" s="11" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>VALOR</t>
         </is>
       </c>
-      <c r="D28" s="11" t="inlineStr">
+      <c r="D29" s="11" t="inlineStr">
         <is>
           <t>% DA LÍQUIDA</t>
         </is>
       </c>
-      <c r="E28" s="11" t="inlineStr">
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>PAGO</t>
         </is>
       </c>
-      <c r="F28" s="11" t="inlineStr">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t>A PAGAR</t>
         </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="12">
-        <f>IF(AREAS!$A$2="","",AREAS!$A$2)</f>
-        <v/>
-      </c>
-      <c r="C29" s="13">
-        <f>IF(B29="","",SUMIF(SAIDAS!$B$6:$B$500,B29,SAIDAS!$G$6:$G$500))</f>
-        <v/>
-      </c>
-      <c r="D29" s="21">
-        <f>IF(OR(B29="",$C$25=0),"",C29/$C$25)</f>
-        <v/>
-      </c>
-      <c r="E29" s="13">
-        <f>IF(B29="","",SUMIFS(SAIDAS!$G$6:$G$500,SAIDAS!$B$6:$B$500,B29,SAIDAS!$H$6:$H$500,"PAGO"))</f>
-        <v/>
-      </c>
-      <c r="F29" s="13">
-        <f>IF(B29="","",C29-E29)</f>
-        <v/>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="12">
-        <f>IF(AREAS!$A$3="","",AREAS!$A$3)</f>
+        <f>IF(AREAS!$A$2="","",AREAS!$A$2)</f>
         <v/>
       </c>
       <c r="C30" s="13">
@@ -1010,7 +1005,7 @@
         <v/>
       </c>
       <c r="D30" s="21">
-        <f>IF(OR(B30="",$C$25=0),"",C30/$C$25)</f>
+        <f>IF(OR(B30="",$C$26=0),"",C30/$C$26)</f>
         <v/>
       </c>
       <c r="E30" s="13">
@@ -1024,7 +1019,7 @@
     </row>
     <row r="31">
       <c r="B31" s="12">
-        <f>IF(AREAS!$A$4="","",AREAS!$A$4)</f>
+        <f>IF(AREAS!$A$3="","",AREAS!$A$3)</f>
         <v/>
       </c>
       <c r="C31" s="13">
@@ -1032,7 +1027,7 @@
         <v/>
       </c>
       <c r="D31" s="21">
-        <f>IF(OR(B31="",$C$25=0),"",C31/$C$25)</f>
+        <f>IF(OR(B31="",$C$26=0),"",C31/$C$26)</f>
         <v/>
       </c>
       <c r="E31" s="13">
@@ -1046,7 +1041,7 @@
     </row>
     <row r="32">
       <c r="B32" s="12">
-        <f>IF(AREAS!$A$5="","",AREAS!$A$5)</f>
+        <f>IF(AREAS!$A$4="","",AREAS!$A$4)</f>
         <v/>
       </c>
       <c r="C32" s="13">
@@ -1054,7 +1049,7 @@
         <v/>
       </c>
       <c r="D32" s="21">
-        <f>IF(OR(B32="",$C$25=0),"",C32/$C$25)</f>
+        <f>IF(OR(B32="",$C$26=0),"",C32/$C$26)</f>
         <v/>
       </c>
       <c r="E32" s="13">
@@ -1068,7 +1063,7 @@
     </row>
     <row r="33">
       <c r="B33" s="12">
-        <f>IF(AREAS!$A$6="","",AREAS!$A$6)</f>
+        <f>IF(AREAS!$A$5="","",AREAS!$A$5)</f>
         <v/>
       </c>
       <c r="C33" s="13">
@@ -1076,7 +1071,7 @@
         <v/>
       </c>
       <c r="D33" s="21">
-        <f>IF(OR(B33="",$C$25=0),"",C33/$C$25)</f>
+        <f>IF(OR(B33="",$C$26=0),"",C33/$C$26)</f>
         <v/>
       </c>
       <c r="E33" s="13">
@@ -1090,7 +1085,7 @@
     </row>
     <row r="34">
       <c r="B34" s="12">
-        <f>IF(AREAS!$A$7="","",AREAS!$A$7)</f>
+        <f>IF(AREAS!$A$6="","",AREAS!$A$6)</f>
         <v/>
       </c>
       <c r="C34" s="13">
@@ -1098,7 +1093,7 @@
         <v/>
       </c>
       <c r="D34" s="21">
-        <f>IF(OR(B34="",$C$25=0),"",C34/$C$25)</f>
+        <f>IF(OR(B34="",$C$26=0),"",C34/$C$26)</f>
         <v/>
       </c>
       <c r="E34" s="13">
@@ -1112,7 +1107,7 @@
     </row>
     <row r="35">
       <c r="B35" s="12">
-        <f>IF(AREAS!$A$8="","",AREAS!$A$8)</f>
+        <f>IF(AREAS!$A$7="","",AREAS!$A$7)</f>
         <v/>
       </c>
       <c r="C35" s="13">
@@ -1120,7 +1115,7 @@
         <v/>
       </c>
       <c r="D35" s="21">
-        <f>IF(OR(B35="",$C$25=0),"",C35/$C$25)</f>
+        <f>IF(OR(B35="",$C$26=0),"",C35/$C$26)</f>
         <v/>
       </c>
       <c r="E35" s="13">
@@ -1134,7 +1129,7 @@
     </row>
     <row r="36">
       <c r="B36" s="12">
-        <f>IF(AREAS!$A$9="","",AREAS!$A$9)</f>
+        <f>IF(AREAS!$A$8="","",AREAS!$A$8)</f>
         <v/>
       </c>
       <c r="C36" s="13">
@@ -1142,7 +1137,7 @@
         <v/>
       </c>
       <c r="D36" s="21">
-        <f>IF(OR(B36="",$C$25=0),"",C36/$C$25)</f>
+        <f>IF(OR(B36="",$C$26=0),"",C36/$C$26)</f>
         <v/>
       </c>
       <c r="E36" s="13">
@@ -1156,7 +1151,7 @@
     </row>
     <row r="37">
       <c r="B37" s="12">
-        <f>IF(AREAS!$A$10="","",AREAS!$A$10)</f>
+        <f>IF(AREAS!$A$9="","",AREAS!$A$9)</f>
         <v/>
       </c>
       <c r="C37" s="13">
@@ -1164,7 +1159,7 @@
         <v/>
       </c>
       <c r="D37" s="21">
-        <f>IF(OR(B37="",$C$25=0),"",C37/$C$25)</f>
+        <f>IF(OR(B37="",$C$26=0),"",C37/$C$26)</f>
         <v/>
       </c>
       <c r="E37" s="13">
@@ -1178,7 +1173,7 @@
     </row>
     <row r="38">
       <c r="B38" s="12">
-        <f>IF(AREAS!$A$11="","",AREAS!$A$11)</f>
+        <f>IF(AREAS!$A$10="","",AREAS!$A$10)</f>
         <v/>
       </c>
       <c r="C38" s="13">
@@ -1186,7 +1181,7 @@
         <v/>
       </c>
       <c r="D38" s="21">
-        <f>IF(OR(B38="",$C$25=0),"",C38/$C$25)</f>
+        <f>IF(OR(B38="",$C$26=0),"",C38/$C$26)</f>
         <v/>
       </c>
       <c r="E38" s="13">
@@ -1200,7 +1195,7 @@
     </row>
     <row r="39">
       <c r="B39" s="12">
-        <f>IF(AREAS!$A$12="","",AREAS!$A$12)</f>
+        <f>IF(AREAS!$A$11="","",AREAS!$A$11)</f>
         <v/>
       </c>
       <c r="C39" s="13">
@@ -1208,7 +1203,7 @@
         <v/>
       </c>
       <c r="D39" s="21">
-        <f>IF(OR(B39="",$C$25=0),"",C39/$C$25)</f>
+        <f>IF(OR(B39="",$C$26=0),"",C39/$C$26)</f>
         <v/>
       </c>
       <c r="E39" s="13">
@@ -1222,7 +1217,7 @@
     </row>
     <row r="40">
       <c r="B40" s="12">
-        <f>IF(AREAS!$A$13="","",AREAS!$A$13)</f>
+        <f>IF(AREAS!$A$12="","",AREAS!$A$12)</f>
         <v/>
       </c>
       <c r="C40" s="13">
@@ -1230,7 +1225,7 @@
         <v/>
       </c>
       <c r="D40" s="21">
-        <f>IF(OR(B40="",$C$25=0),"",C40/$C$25)</f>
+        <f>IF(OR(B40="",$C$26=0),"",C40/$C$26)</f>
         <v/>
       </c>
       <c r="E40" s="13">
@@ -1244,7 +1239,7 @@
     </row>
     <row r="41">
       <c r="B41" s="12">
-        <f>IF(AREAS!$A$14="","",AREAS!$A$14)</f>
+        <f>IF(AREAS!$A$13="","",AREAS!$A$13)</f>
         <v/>
       </c>
       <c r="C41" s="13">
@@ -1252,7 +1247,7 @@
         <v/>
       </c>
       <c r="D41" s="21">
-        <f>IF(OR(B41="",$C$25=0),"",C41/$C$25)</f>
+        <f>IF(OR(B41="",$C$26=0),"",C41/$C$26)</f>
         <v/>
       </c>
       <c r="E41" s="13">
@@ -1265,145 +1260,167 @@
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B42" s="12">
+        <f>IF(AREAS!$A$14="","",AREAS!$A$14)</f>
+        <v/>
+      </c>
+      <c r="C42" s="13">
+        <f>IF(B42="","",SUMIF(SAIDAS!$B$6:$B$500,B42,SAIDAS!$G$6:$G$500))</f>
+        <v/>
+      </c>
+      <c r="D42" s="21">
+        <f>IF(OR(B42="",$C$26=0),"",C42/$C$26)</f>
+        <v/>
+      </c>
+      <c r="E42" s="13">
+        <f>IF(B42="","",SUMIFS(SAIDAS!$G$6:$G$500,SAIDAS!$B$6:$B$500,B42,SAIDAS!$H$6:$H$500,"PAGO"))</f>
+        <v/>
+      </c>
+      <c r="F42" s="13">
+        <f>IF(B42="","",C42-E42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="22" t="inlineStr">
         <is>
           <t>SEM ÁREA — classificar na aba SAÍDAS</t>
         </is>
       </c>
-      <c r="C42" s="13">
-        <f>ROUND(SUM(SAIDAS!$G$6:$G$500)-SUM(C29:C41),2)</f>
-        <v/>
-      </c>
-      <c r="D42" s="21" t="n"/>
-      <c r="E42" s="13" t="n"/>
-      <c r="F42" s="13" t="n"/>
-    </row>
-    <row r="43">
-      <c r="B43" s="23" t="inlineStr">
+      <c r="C43" s="13">
+        <f>ROUND(SUM(SAIDAS!$G$6:$G$500)-SUM(C30:C42),2)</f>
+        <v/>
+      </c>
+      <c r="D43" s="21" t="n"/>
+      <c r="E43" s="13" t="n"/>
+      <c r="F43" s="13" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="23" t="inlineStr">
         <is>
           <t>TOTAL SAÍDAS</t>
         </is>
       </c>
-      <c r="C43" s="24">
+      <c r="C44" s="24">
         <f>ROUND(SUM(SAIDAS!$G$6:$G$500),2)</f>
         <v/>
       </c>
-      <c r="D43" s="25">
-        <f>IF($C$25=0,"",C43/$C$25)</f>
-        <v/>
-      </c>
-      <c r="E43" s="24">
+      <c r="D44" s="25">
+        <f>IF($C$26=0,"",C44/$C$26)</f>
+        <v/>
+      </c>
+      <c r="E44" s="24">
         <f>SUMIF(SAIDAS!$H$6:$H$500,"PAGO",SAIDAS!$G$6:$G$500)</f>
         <v/>
       </c>
-      <c r="F43" s="24">
-        <f>C43-E43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="B45" s="10" t="inlineStr">
+      <c r="F44" s="24">
+        <f>C44-E44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="B46" s="10" t="inlineStr">
         <is>
           <t>3.  RESULTADO</t>
         </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>ENTRADA LÍQUIDA</t>
-        </is>
-      </c>
-      <c r="C46" s="13">
-        <f>C25</f>
-        <v/>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="12" t="inlineStr">
         <is>
+          <t>ENTRADA LÍQUIDA</t>
+        </is>
+      </c>
+      <c r="C47" s="13">
+        <f>C26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
           <t>(−) TOTAL SAÍDAS</t>
         </is>
       </c>
-      <c r="C47" s="13">
-        <f>C43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" ht="24" customHeight="1">
-      <c r="B48" s="26" t="inlineStr">
+      <c r="C48" s="13">
+        <f>C44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="24" customHeight="1">
+      <c r="B49" s="26" t="inlineStr">
         <is>
           <t>(=) LUCRO DA YAD</t>
         </is>
       </c>
-      <c r="C48" s="27">
-        <f>C25-C43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="12" t="inlineStr">
+      <c r="C49" s="27">
+        <f>C26-C44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>MARGEM (sobre a entrada bruta)</t>
         </is>
       </c>
-      <c r="C49" s="28">
-        <f>IF(C22=0,"",C48/C22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="B51" s="10" t="inlineStr">
+      <c r="C50" s="28">
+        <f>IF(C23=0,"",C49/C23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="B52" s="10" t="inlineStr">
         <is>
           <t>4.  CAIXA — o que já andou e o que falta</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="28" customHeight="1">
-      <c r="B52" s="11" t="inlineStr"/>
-      <c r="C52" s="11" t="inlineStr">
+    <row r="53" ht="28" customHeight="1">
+      <c r="B53" s="11" t="inlineStr"/>
+      <c r="C53" s="11" t="inlineStr">
         <is>
           <t>JÁ ANDOU</t>
         </is>
       </c>
-      <c r="D52" s="11" t="inlineStr">
+      <c r="D53" s="11" t="inlineStr">
         <is>
           <t>FALTA</t>
         </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>ENTRADAS (recebido / a receber)</t>
-        </is>
-      </c>
-      <c r="C53" s="13">
-        <f>SUMIF(E17:E21,"RECEBIDO",C17:C21)</f>
-        <v/>
-      </c>
-      <c r="D53" s="13">
-        <f>C22-C53</f>
-        <v/>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="12" t="inlineStr">
         <is>
+          <t>ENTRADAS (recebido / a receber)</t>
+        </is>
+      </c>
+      <c r="C54" s="13">
+        <f>SUMIF(E17:E22,"RECEBIDO",C17:C22)</f>
+        <v/>
+      </c>
+      <c r="D54" s="13">
+        <f>C23-C54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
           <t>SAÍDAS (pago / a pagar)</t>
         </is>
       </c>
-      <c r="C54" s="13">
-        <f>E43</f>
-        <v/>
-      </c>
-      <c r="D54" s="13">
-        <f>F43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="B56" s="29" t="inlineStr">
+      <c r="C55" s="13">
+        <f>E44</f>
+        <v/>
+      </c>
+      <c r="D55" s="13">
+        <f>F44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="29" t="inlineStr">
         <is>
           <t>Preencha só a aba SAIDAS — esta aqui é toda fórmula. Célula amarela é campo para digitar.</t>
         </is>
@@ -1411,27 +1428,27 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B56:F56"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="C3:F3"/>
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B51:F51"/>
-    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B28:F28"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B46:F46"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="C2:F2"/>
     <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B57:F57"/>
+    <mergeCell ref="B52:F52"/>
   </mergeCells>
-  <conditionalFormatting sqref="C42">
+  <conditionalFormatting sqref="C43">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.005</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B48:C48">
+  <conditionalFormatting sqref="B49:C49">
     <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
@@ -1440,7 +1457,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E17:E21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E17:E22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A RECEBER,RECEBIDO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1671,7 +1688,7 @@
         <v>10</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="G6" s="35">
         <f>IF(OR(E6="",F6=""),"",ROUND(E6*F6,2))</f>
@@ -1683,11 +1700,7 @@
         </is>
       </c>
       <c r="I6" s="14" t="n"/>
-      <c r="J6" s="12" t="inlineStr">
-        <is>
-          <t>diária de referência do orçamento — confirmar o combinado</t>
-        </is>
-      </c>
+      <c r="J6" s="12" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="12" t="inlineStr">
@@ -1706,10 +1719,10 @@
         </is>
       </c>
       <c r="E7" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="G7" s="35">
         <f>IF(OR(E7="",F7=""),"",ROUND(E7*F7,2))</f>
@@ -1721,11 +1734,7 @@
         </is>
       </c>
       <c r="I7" s="14" t="n"/>
-      <c r="J7" s="12" t="inlineStr">
-        <is>
-          <t>diária de referência do orçamento — confirmar o combinado</t>
-        </is>
-      </c>
+      <c r="J7" s="12" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="B8" s="12" t="inlineStr">
@@ -1744,7 +1753,7 @@
         </is>
       </c>
       <c r="E8" s="15" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F8" s="13" t="n">
         <v>800</v>
@@ -1759,11 +1768,7 @@
         </is>
       </c>
       <c r="I8" s="14" t="n"/>
-      <c r="J8" s="12" t="inlineStr">
-        <is>
-          <t>diária de referência do orçamento — confirmar o combinado</t>
-        </is>
-      </c>
+      <c r="J8" s="12" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="B9" s="12" t="inlineStr">
@@ -1782,7 +1787,7 @@
         </is>
       </c>
       <c r="E9" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F9" s="13" t="n">
         <v>500</v>
@@ -1797,11 +1802,7 @@
         </is>
       </c>
       <c r="I9" s="14" t="n"/>
-      <c r="J9" s="12" t="inlineStr">
-        <is>
-          <t>diária de referência do orçamento — confirmar o combinado</t>
-        </is>
-      </c>
+      <c r="J9" s="12" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="B10" s="12" t="inlineStr">
@@ -1820,7 +1821,7 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F10" s="13" t="n">
         <v>500</v>
@@ -1835,11 +1836,7 @@
         </is>
       </c>
       <c r="I10" s="14" t="n"/>
-      <c r="J10" s="12" t="inlineStr">
-        <is>
-          <t>diária de referência do orçamento — confirmar o combinado</t>
-        </is>
-      </c>
+      <c r="J10" s="12" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="B11" s="12" t="inlineStr">
@@ -1858,7 +1855,7 @@
         </is>
       </c>
       <c r="E11" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F11" s="13" t="n">
         <v>500</v>
@@ -1873,11 +1870,7 @@
         </is>
       </c>
       <c r="I11" s="14" t="n"/>
-      <c r="J11" s="12" t="inlineStr">
-        <is>
-          <t>diária de referência do orçamento — confirmar o combinado</t>
-        </is>
-      </c>
+      <c r="J11" s="12" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="B12" s="12" t="inlineStr">
@@ -1911,11 +1904,7 @@
         </is>
       </c>
       <c r="I12" s="14" t="n"/>
-      <c r="J12" s="12" t="inlineStr">
-        <is>
-          <t>diária de referência do orçamento — confirmar o combinado</t>
-        </is>
-      </c>
+      <c r="J12" s="12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="12" t="inlineStr">
@@ -1949,11 +1938,7 @@
         </is>
       </c>
       <c r="I13" s="14" t="n"/>
-      <c r="J13" s="12" t="inlineStr">
-        <is>
-          <t>diária de referência do orçamento — confirmar o combinado</t>
-        </is>
-      </c>
+      <c r="J13" s="12" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="12" t="inlineStr">
@@ -1992,23 +1977,25 @@
     <row r="15">
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>TRANSPORTE E LOGÍSTICA</t>
+          <t>EQUIPE</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Combustível — caminhão de equipamento</t>
+          <t>Larissa</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>SP ↔ Barretos, ida e volta</t>
+          <t>Produção Adm</t>
         </is>
       </c>
       <c r="E15" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="16" t="n"/>
+      <c r="F15" s="13" t="n">
+        <v>2500</v>
+      </c>
       <c r="G15" s="35">
         <f>IF(OR(E15="",F15=""),"",ROUND(E15*F15,2))</f>
         <v/>
@@ -2029,18 +2016,20 @@
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Combustível — carro de apoio</t>
+          <t>Combustível — caminhão de equipamento</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>equipe</t>
+          <t>SP ↔ Barretos, ida e volta</t>
         </is>
       </c>
       <c r="E16" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="16" t="n"/>
+      <c r="F16" s="13" t="n">
+        <v>2000</v>
+      </c>
       <c r="G16" s="35">
         <f>IF(OR(E16="",F16=""),"",ROUND(E16*F16,2))</f>
         <v/>
@@ -2061,18 +2050,20 @@
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Pedágio</t>
+          <t>Combustível — carro de apoio</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>ida e volta</t>
+          <t>equipe</t>
         </is>
       </c>
       <c r="E17" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="16" t="n"/>
+      <c r="F17" s="13" t="n">
+        <v>1000</v>
+      </c>
       <c r="G17" s="35">
         <f>IF(OR(E17="",F17=""),"",ROUND(E17*F17,2))</f>
         <v/>
@@ -2088,23 +2079,25 @@
     <row r="18">
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>ALIMENTAÇÃO</t>
+          <t>TRANSPORTE E LOGÍSTICA</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>Alimentação na estrada — ida</t>
+          <t>Pedágio</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>equipe</t>
+          <t>ida e volta</t>
         </is>
       </c>
       <c r="E18" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F18" s="16" t="n"/>
+      <c r="F18" s="13" t="n">
+        <v>400</v>
+      </c>
       <c r="G18" s="35">
         <f>IF(OR(E18="",F18=""),"",ROUND(E18*F18,2))</f>
         <v/>
@@ -2125,7 +2118,7 @@
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Alimentação na estrada — volta</t>
+          <t>Alimentação na estrada — ida</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -2136,7 +2129,9 @@
       <c r="E19" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="16" t="n"/>
+      <c r="F19" s="13" t="n">
+        <v>500</v>
+      </c>
       <c r="G19" s="35">
         <f>IF(OR(E19="",F19=""),"",ROUND(E19*F19,2))</f>
         <v/>
@@ -2157,16 +2152,20 @@
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>Alimentação da equipe durante o evento</t>
+          <t>Alimentação na estrada — volta</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>8 pessoas × diárias</t>
-        </is>
-      </c>
-      <c r="E20" s="36" t="n"/>
-      <c r="F20" s="16" t="n"/>
+          <t>equipe</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>500</v>
+      </c>
       <c r="G20" s="35">
         <f>IF(OR(E20="",F20=""),"",ROUND(E20*F20,2))</f>
         <v/>
@@ -2177,30 +2176,30 @@
         </is>
       </c>
       <c r="I20" s="14" t="n"/>
-      <c r="J20" s="12" t="inlineStr">
-        <is>
-          <t>checar o que o Clube do Cowboy cobre de catering</t>
-        </is>
-      </c>
+      <c r="J20" s="12" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>HOSPEDAGEM</t>
+          <t>ALIMENTAÇÃO</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Hospedagem da equipe em Barretos</t>
+          <t>Alimentação da equipe durante o evento</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>diárias × quartos</t>
-        </is>
-      </c>
-      <c r="E21" s="36" t="n"/>
-      <c r="F21" s="16" t="n"/>
+          <t>8 pessoas × diárias</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="F21" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="G21" s="35">
         <f>IF(OR(E21="",F21=""),"",ROUND(E21*F21,2))</f>
         <v/>
@@ -2213,31 +2212,31 @@
       <c r="I21" s="14" t="n"/>
       <c r="J21" s="12" t="inlineStr">
         <is>
-          <t>confirmar se é por conta do cliente</t>
+          <t>checar o que o Clube do Cowboy cobre de catering</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>EQUIPAMENTO E MANUTENÇÃO</t>
+          <t>HOSPEDAGEM</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>Conserto do caminhão</t>
+          <t>Hospedagem da equipe em Barretos</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>caminhão que leva o equipamento</t>
+          <t>diárias × quartos</t>
         </is>
       </c>
       <c r="E22" s="15" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F22" s="13" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="G22" s="35">
         <f>IF(OR(E22="",F22=""),"",ROUND(E22*F22,2))</f>
@@ -2251,37 +2250,81 @@
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="12" t="inlineStr">
         <is>
-          <t>valor aproximado informado pela produção</t>
+          <t>confirmar se é por conta do cliente</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="12" t="n"/>
-      <c r="C23" s="12" t="n"/>
-      <c r="D23" s="12" t="n"/>
-      <c r="E23" s="36" t="n"/>
-      <c r="F23" s="16" t="n"/>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>EQUIPAMENTO E MANUTENÇÃO</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Conserto do caminhão</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Caminhão que leva o equipamento</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="13" t="n">
+        <v>1500</v>
+      </c>
       <c r="G23" s="35">
         <f>IF(OR(E23="",F23=""),"",ROUND(E23*F23,2))</f>
         <v/>
       </c>
-      <c r="H23" s="15" t="n"/>
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>A PAGAR</t>
+        </is>
+      </c>
       <c r="I23" s="14" t="n"/>
-      <c r="J23" s="12" t="n"/>
+      <c r="J23" s="12" t="inlineStr">
+        <is>
+          <t>valor aproximado informado pela produção</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="36" t="n"/>
-      <c r="F24" s="16" t="n"/>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>LOCAÇÃO DE TERCEIROS</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Danilo</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Cameras Broadcast</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>1000</v>
+      </c>
       <c r="G24" s="35">
         <f>IF(OR(E24="",F24=""),"",ROUND(E24*F24,2))</f>
         <v/>
       </c>
-      <c r="H24" s="15" t="n"/>
+      <c r="H24" s="15" t="inlineStr">
+        <is>
+          <t>A PAGAR</t>
+        </is>
+      </c>
       <c r="I24" s="14" t="n"/>
-      <c r="J24" s="12" t="n"/>
+      <c r="J24" s="12" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="B25" s="12" t="n"/>

</xml_diff>

<commit_message>
producao: Barretos 2026 v3 — alimentação no local por conta do cliente
O Clube do Cowboy fornece a alimentação no local. A linha continua em zero,
mas agora zero por não ser custo, e não por faltar preencher — status vazio
(nada a pagar) e a observação registrando quem cobre. Alimentação na estrada
segue por conta da YAD.

Nenhum total muda: bruto 108.500, líquida 91.140, saídas 55.400, lucro
35.740. O que muda é a planilha parar de sinalizar pendência onde não há.

Hospedagem segue como a única linha em aberto — por isso a situação continua
EM ANDAMENTO.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NubHinCg53tN7sLp5QNqJV
</commit_message>
<xml_diff>
--- a/producao/pressupostos/PRESSUPOSTO_REAL_BARRETOS_2026.xlsx
+++ b/producao/pressupostos/PRESSUPOSTO_REAL_BARRETOS_2026.xlsx
@@ -785,7 +785,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D13" s="8" t="n"/>
@@ -2191,7 +2191,7 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>8 pessoas × diárias</t>
+          <t>no local, durante o evento</t>
         </is>
       </c>
       <c r="E21" s="15" t="n">
@@ -2204,15 +2204,11 @@
         <f>IF(OR(E21="",F21=""),"",ROUND(E21*F21,2))</f>
         <v/>
       </c>
-      <c r="H21" s="15" t="inlineStr">
-        <is>
-          <t>A PAGAR</t>
-        </is>
-      </c>
+      <c r="H21" s="15" t="inlineStr"/>
       <c r="I21" s="14" t="n"/>
       <c r="J21" s="12" t="inlineStr">
         <is>
-          <t>checar o que o Clube do Cowboy cobre de catering</t>
+          <t>CLUBE DO COWBOY fornece no local — sem custo para a YAD</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
producao: Barretos 2026 v4 — pressuposto fechado
Hospedagem também é por conta do Clube do Cowboy. Com isso não sobra linha
em aberto e a situação vai para FECHADO.

Bruto 108.500 · imposto 16% 17.360 · líquida 91.140 · saídas 55.400 ·
lucro 35.740 (32,9%). Nenhum total muda desde a v2 — as duas últimas
revisões só resolveram o que estava indefinido.

Vira gotcha na nota: zero por não ser custo e zero por faltar preencher
somam igual e significam o oposto. O que separa é o STATUS — linha coberta
pelo cliente fica sem status, com a OBS dizendo quem cobre.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NubHinCg53tN7sLp5QNqJV
</commit_message>
<xml_diff>
--- a/producao/pressupostos/PRESSUPOSTO_REAL_BARRETOS_2026.xlsx
+++ b/producao/pressupostos/PRESSUPOSTO_REAL_BARRETOS_2026.xlsx
@@ -785,7 +785,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v4</t>
         </is>
       </c>
       <c r="D13" s="8" t="n"/>
@@ -796,7 +796,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>EM ANDAMENTO</t>
+          <t>FECHADO</t>
         </is>
       </c>
     </row>
@@ -2225,7 +2225,7 @@
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>diárias × quartos</t>
+          <t>no local, durante o evento</t>
         </is>
       </c>
       <c r="E22" s="15" t="n">
@@ -2238,15 +2238,11 @@
         <f>IF(OR(E22="",F22=""),"",ROUND(E22*F22,2))</f>
         <v/>
       </c>
-      <c r="H22" s="15" t="inlineStr">
-        <is>
-          <t>A PAGAR</t>
-        </is>
-      </c>
+      <c r="H22" s="15" t="inlineStr"/>
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="12" t="inlineStr">
         <is>
-          <t>confirmar se é por conta do cliente</t>
+          <t>CLUBE DO COWBOY fornece — sem custo para a YAD</t>
         </is>
       </c>
     </row>

</xml_diff>